<commit_message>
Add RP7.4 .docx report, input dataset and data-driven calculation code
- RP7.4 report in .docx (house style RP7.3: header progetto, 4 sezioni, tabelle
  con intestazioni verdi, figure integrate).
- RP7.4_dataset_sintetico.xlsx: dataset di input pulito e editabile (una riga per
  tipologia x periodo t/t-1), da sostituire con i dati reali a fine progetto.
- RP7.4_build.py rifattorizzato: legge il dataset (o lo crea dai default),
  ricostruisce indicatori/indici/figure -> workflow "sostituisci e rilancia";
  numeri invariati (P-TSI_z T3>T1>T2; CR=0.0079). Aggiunto RP7.4_make_docx.py.
- Rimosso RP7.4_data_collection.xlsx (superato dal dataset di input).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TDWdb7nMyYxCAQNw9GyeGc
</commit_message>
<xml_diff>
--- a/RP7.4_calculation_log.xlsx
+++ b/RP7.4_calculation_log.xlsx
@@ -434,11 +434,11 @@
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="42" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
@@ -532,7 +532,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>IOA_SCR_input</t>
+          <t>dataset:INPUT</t>
         </is>
       </c>
       <c r="H2" t="n">
@@ -587,7 +587,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>IOA_SCR_input</t>
+          <t>dataset:INPUT</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -642,7 +642,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>IOA_SCR_input</t>
+          <t>dataset:INPUT</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -697,7 +697,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>IOA_SCR_input</t>
+          <t>dataset:INPUT</t>
         </is>
       </c>
       <c r="H5" t="n">
@@ -752,7 +752,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>IOA_SCR_input</t>
+          <t>dataset:INPUT</t>
         </is>
       </c>
       <c r="H6" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>IOA_SCR_input</t>
+          <t>dataset:INPUT</t>
         </is>
       </c>
       <c r="H7" t="n">
@@ -862,7 +862,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>IOA_SCR_input</t>
+          <t>dataset:INPUT</t>
         </is>
       </c>
       <c r="H8" t="n">
@@ -917,7 +917,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>IOA_SCR_input</t>
+          <t>dataset:INPUT</t>
         </is>
       </c>
       <c r="H9" t="n">
@@ -972,7 +972,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>IOA_SCR_input</t>
+          <t>dataset:INPUT</t>
         </is>
       </c>
       <c r="H10" t="n">
@@ -1027,7 +1027,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>OP_PsI_input</t>
+          <t>dataset:INPUT</t>
         </is>
       </c>
       <c r="H11" t="n">
@@ -1082,7 +1082,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>OP_PsI_input</t>
+          <t>dataset:INPUT</t>
         </is>
       </c>
       <c r="H12" t="n">
@@ -1137,7 +1137,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>OP_PsI_input</t>
+          <t>dataset:INPUT</t>
         </is>
       </c>
       <c r="H13" t="n">
@@ -1192,7 +1192,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>OP_PsI_input</t>
+          <t>dataset:INPUT</t>
         </is>
       </c>
       <c r="H14" t="n">
@@ -1247,7 +1247,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>OP_PsI_input</t>
+          <t>dataset:INPUT</t>
         </is>
       </c>
       <c r="H15" t="n">
@@ -1302,7 +1302,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>OP_PsI_input</t>
+          <t>dataset:INPUT</t>
         </is>
       </c>
       <c r="H16" t="n">
@@ -1357,7 +1357,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>OP_PsI_input</t>
+          <t>dataset:INPUT</t>
         </is>
       </c>
       <c r="H17" t="n">
@@ -1412,7 +1412,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>OP_PsI_input</t>
+          <t>dataset:INPUT</t>
         </is>
       </c>
       <c r="H18" t="n">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>OP_PsI_input</t>
+          <t>dataset:INPUT</t>
         </is>
       </c>
       <c r="H19" t="n">
@@ -1522,7 +1522,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>TQ_OCR_input</t>
+          <t>dataset:INPUT</t>
         </is>
       </c>
       <c r="H20" t="n">
@@ -1577,7 +1577,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>TQ_OCR_input</t>
+          <t>dataset:INPUT</t>
         </is>
       </c>
       <c r="H21" t="n">
@@ -1632,7 +1632,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>TQ_OCR_input</t>
+          <t>dataset:INPUT</t>
         </is>
       </c>
       <c r="H22" t="n">
@@ -1687,7 +1687,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>TQ_OCR_input</t>
+          <t>dataset:INPUT</t>
         </is>
       </c>
       <c r="H23" t="n">
@@ -1742,7 +1742,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>TQ_OCR_input</t>
+          <t>dataset:INPUT</t>
         </is>
       </c>
       <c r="H24" t="n">
@@ -1797,7 +1797,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>TQ_OCR_input</t>
+          <t>dataset:INPUT</t>
         </is>
       </c>
       <c r="H25" t="n">
@@ -1852,7 +1852,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>TQ_OCR_input</t>
+          <t>dataset:INPUT</t>
         </is>
       </c>
       <c r="H26" t="n">
@@ -1907,7 +1907,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>TQ_OCR_input</t>
+          <t>dataset:INPUT</t>
         </is>
       </c>
       <c r="H27" t="n">
@@ -1962,7 +1962,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>TQ_OCR_input</t>
+          <t>dataset:INPUT</t>
         </is>
       </c>
       <c r="H28" t="n">
@@ -3651,14 +3651,14 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Serie 2023-2024 sintetiche provvisorie, ancorate a EPD e serie RP6.x/RP7.3, in corso di consolidamento.</t>
+          <t>Serie 2023-2024 provvisorie, in corso di consolidamento, ancorate a EPD e serie RP6.x/RP7.3.</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>A fine progetto: assessment rieseguito con dati reali, struttura di calcolo invariata.</t>
+          <t>A fine progetto: sostituire i dati nel dataset e rieseguire; struttura di calcolo invariata.</t>
         </is>
       </c>
     </row>

</xml_diff>